<commit_message>
Price check: EUR 1773 (available) 2026-09-17
Co-authored-by: woutergroeneweg-blip <woutergroeneweg-blip@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/prices.xlsx
+++ b/prices.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price History" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Price History" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -138,14 +138,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -168,26 +167,26 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <cat>
             <numRef>
-              <f>'Price History'!$A$2</f>
+              <f>'Price History'!$A$2:$A$13</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Price History'!$B$2</f>
+              <f>'Price History'!$B$2:$B$13</f>
             </numRef>
           </val>
         </ser>
@@ -203,8 +202,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -230,8 +229,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -257,7 +256,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -272,9 +271,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -572,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -658,6 +657,380 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>Baseline from Roompot confirmation screenshot; replace/extend with live automation runs</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-01T11:09:16+02:00</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1809</v>
+      </c>
+      <c r="D3" t="n">
+        <v>95</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>-17</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-05T11:06:27+02:00</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1797</v>
+      </c>
+      <c r="D4" t="n">
+        <v>95</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>-12</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-09T11:06:32+02:00</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1910</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1815</v>
+      </c>
+      <c r="D5" t="n">
+        <v>95</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>+18</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-13T11:11:58+02:00</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1921</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1826</v>
+      </c>
+      <c r="D6" t="n">
+        <v>95</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>+11</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-21T11:05:50+02:00</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1745</v>
+      </c>
+      <c r="D7" t="n">
+        <v>95</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>-81</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-25T11:07:23+02:00</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1844</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1749</v>
+      </c>
+      <c r="D8" t="n">
+        <v>95</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>+4</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-29T11:15:29+02:00</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1876</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1781</v>
+      </c>
+      <c r="D9" t="n">
+        <v>95</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>+32</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-01T11:07:41+02:00</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1767</v>
+      </c>
+      <c r="D10" t="n">
+        <v>95</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>-14</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-05T11:06:59+02:00</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1682</v>
+      </c>
+      <c r="D11" t="n">
+        <v>95</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>-85</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-09T11:08:10+02:00</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1666</v>
+      </c>
+      <c r="D12" t="n">
+        <v>95</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>-16</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:14:39+02:00</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D13" t="n">
+        <v>95</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>+12</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Price check: EUR 1773 (available) 2026-09-21
Co-authored-by: woutergroeneweg-blip <woutergroeneweg-blip@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/prices.xlsx
+++ b/prices.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price History" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Price History" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -138,14 +138,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -168,26 +167,26 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <cat>
             <numRef>
-              <f>'Price History'!$A$2</f>
+              <f>'Price History'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Price History'!$B$2</f>
+              <f>'Price History'!$B$2:$B$14</f>
             </numRef>
           </val>
         </ser>
@@ -203,8 +202,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -230,8 +229,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -257,7 +256,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -272,9 +271,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -572,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -658,6 +657,414 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>Baseline from Roompot confirmation screenshot; replace/extend with live automation runs</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-01T11:09:16+02:00</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1809</v>
+      </c>
+      <c r="D3" t="n">
+        <v>95</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>-17</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-05T11:06:27+02:00</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1797</v>
+      </c>
+      <c r="D4" t="n">
+        <v>95</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>-12</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-09T11:06:32+02:00</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1910</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1815</v>
+      </c>
+      <c r="D5" t="n">
+        <v>95</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>+18</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-13T11:11:58+02:00</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1921</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1826</v>
+      </c>
+      <c r="D6" t="n">
+        <v>95</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>+11</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-21T11:05:50+02:00</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1745</v>
+      </c>
+      <c r="D7" t="n">
+        <v>95</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>-81</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-25T11:07:23+02:00</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1844</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1749</v>
+      </c>
+      <c r="D8" t="n">
+        <v>95</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>+4</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-29T11:15:29+02:00</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1876</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1781</v>
+      </c>
+      <c r="D9" t="n">
+        <v>95</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>+32</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-01T11:07:41+02:00</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1767</v>
+      </c>
+      <c r="D10" t="n">
+        <v>95</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>-14</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-05T11:06:59+02:00</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1682</v>
+      </c>
+      <c r="D11" t="n">
+        <v>95</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>-85</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-09T11:08:10+02:00</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1666</v>
+      </c>
+      <c r="D12" t="n">
+        <v>95</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>-16</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:14:39+02:00</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D13" t="n">
+        <v>95</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>+12</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-21T11:06:05+02:00</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D14" t="n">
+        <v>95</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Price check: EUR 1674 (available) 2026-09-25
Co-authored-by: woutergroeneweg-blip <woutergroeneweg-blip@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/prices.xlsx
+++ b/prices.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price History" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Price History" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -138,14 +138,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -168,26 +167,26 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <cat>
             <numRef>
-              <f>'Price History'!$A$2</f>
+              <f>'Price History'!$A$2:$A$15</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Price History'!$B$2</f>
+              <f>'Price History'!$B$2:$B$15</f>
             </numRef>
           </val>
         </ser>
@@ -203,8 +202,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -230,8 +229,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -257,7 +256,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -272,9 +271,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -572,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -658,6 +657,448 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>Baseline from Roompot confirmation screenshot; replace/extend with live automation runs</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-01T11:09:16+02:00</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1809</v>
+      </c>
+      <c r="D3" t="n">
+        <v>95</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>-17</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-05T11:06:27+02:00</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1797</v>
+      </c>
+      <c r="D4" t="n">
+        <v>95</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>-12</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-09T11:06:32+02:00</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1910</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1815</v>
+      </c>
+      <c r="D5" t="n">
+        <v>95</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>+18</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-13T11:11:58+02:00</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1921</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1826</v>
+      </c>
+      <c r="D6" t="n">
+        <v>95</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>+11</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-21T11:05:50+02:00</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1745</v>
+      </c>
+      <c r="D7" t="n">
+        <v>95</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>-81</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-25T11:07:23+02:00</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1844</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1749</v>
+      </c>
+      <c r="D8" t="n">
+        <v>95</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>+4</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-29T11:15:29+02:00</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1876</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1781</v>
+      </c>
+      <c r="D9" t="n">
+        <v>95</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>+32</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-01T11:07:41+02:00</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1767</v>
+      </c>
+      <c r="D10" t="n">
+        <v>95</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>-14</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-05T11:06:59+02:00</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1682</v>
+      </c>
+      <c r="D11" t="n">
+        <v>95</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>-85</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-09T11:08:10+02:00</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1666</v>
+      </c>
+      <c r="D12" t="n">
+        <v>95</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>-16</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:14:39+02:00</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D13" t="n">
+        <v>95</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>+12</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-21T11:06:05+02:00</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D14" t="n">
+        <v>95</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:09:00+02:00</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1674</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1579</v>
+      </c>
+      <c r="D15" t="n">
+        <v>95</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>-99</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Price check: EUR 1774 (available) 2026-09-29
Co-authored-by: woutergroeneweg-blip <woutergroeneweg-blip@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/prices.xlsx
+++ b/prices.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price History" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Price History" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -138,14 +138,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -168,26 +167,26 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <cat>
             <numRef>
-              <f>'Price History'!$A$2</f>
+              <f>'Price History'!$A$2:$A$16</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Price History'!$B$2</f>
+              <f>'Price History'!$B$2:$B$16</f>
             </numRef>
           </val>
         </ser>
@@ -203,8 +202,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -230,8 +229,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -257,7 +256,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -272,9 +271,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -572,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -658,6 +657,482 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>Baseline from Roompot confirmation screenshot; replace/extend with live automation runs</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-01T11:09:16+02:00</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1809</v>
+      </c>
+      <c r="D3" t="n">
+        <v>95</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>-17</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-05T11:06:27+02:00</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1797</v>
+      </c>
+      <c r="D4" t="n">
+        <v>95</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>-12</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-09T11:06:32+02:00</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1910</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1815</v>
+      </c>
+      <c r="D5" t="n">
+        <v>95</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>+18</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-13T11:11:58+02:00</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1921</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1826</v>
+      </c>
+      <c r="D6" t="n">
+        <v>95</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>+11</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-21T11:05:50+02:00</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1745</v>
+      </c>
+      <c r="D7" t="n">
+        <v>95</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>-81</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-25T11:07:23+02:00</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1844</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1749</v>
+      </c>
+      <c r="D8" t="n">
+        <v>95</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>+4</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-29T11:15:29+02:00</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1876</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1781</v>
+      </c>
+      <c r="D9" t="n">
+        <v>95</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>+32</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-01T11:07:41+02:00</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1767</v>
+      </c>
+      <c r="D10" t="n">
+        <v>95</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>-14</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-05T11:06:59+02:00</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1682</v>
+      </c>
+      <c r="D11" t="n">
+        <v>95</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>-85</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-09T11:08:10+02:00</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1666</v>
+      </c>
+      <c r="D12" t="n">
+        <v>95</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>-16</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:14:39+02:00</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D13" t="n">
+        <v>95</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>+12</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-21T11:06:05+02:00</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D14" t="n">
+        <v>95</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:09:00+02:00</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1674</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1579</v>
+      </c>
+      <c r="D15" t="n">
+        <v>95</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>-99</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29T11:05:58+02:00</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1774</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1679</v>
+      </c>
+      <c r="D16" t="n">
+        <v>95</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Price check: EUR 1749 (available) 2026-10-01
Co-authored-by: woutergroeneweg-blip <woutergroeneweg-blip@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/prices.xlsx
+++ b/prices.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price History" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Price History" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -138,14 +138,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -168,26 +167,26 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <cat>
             <numRef>
-              <f>'Price History'!$A$2</f>
+              <f>'Price History'!$A$2:$A$17</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Price History'!$B$2</f>
+              <f>'Price History'!$B$2:$B$17</f>
             </numRef>
           </val>
         </ser>
@@ -203,8 +202,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -230,8 +229,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -257,7 +256,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -272,9 +271,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -572,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -658,6 +657,516 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>Baseline from Roompot confirmation screenshot; replace/extend with live automation runs</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-01T11:09:16+02:00</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1809</v>
+      </c>
+      <c r="D3" t="n">
+        <v>95</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>-17</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-05T11:06:27+02:00</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1797</v>
+      </c>
+      <c r="D4" t="n">
+        <v>95</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>-12</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-09T11:06:32+02:00</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1910</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1815</v>
+      </c>
+      <c r="D5" t="n">
+        <v>95</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>+18</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-13T11:11:58+02:00</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1921</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1826</v>
+      </c>
+      <c r="D6" t="n">
+        <v>95</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>+11</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-21T11:05:50+02:00</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1745</v>
+      </c>
+      <c r="D7" t="n">
+        <v>95</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>-81</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-25T11:07:23+02:00</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1844</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1749</v>
+      </c>
+      <c r="D8" t="n">
+        <v>95</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>+4</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-29T11:15:29+02:00</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1876</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1781</v>
+      </c>
+      <c r="D9" t="n">
+        <v>95</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>+32</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-01T11:07:41+02:00</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1767</v>
+      </c>
+      <c r="D10" t="n">
+        <v>95</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>-14</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-05T11:06:59+02:00</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1682</v>
+      </c>
+      <c r="D11" t="n">
+        <v>95</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>-85</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-09T11:08:10+02:00</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1666</v>
+      </c>
+      <c r="D12" t="n">
+        <v>95</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>-16</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:14:39+02:00</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D13" t="n">
+        <v>95</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>+12</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-21T11:06:05+02:00</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D14" t="n">
+        <v>95</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:09:00+02:00</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1674</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1579</v>
+      </c>
+      <c r="D15" t="n">
+        <v>95</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>-99</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29T11:05:58+02:00</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1774</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1679</v>
+      </c>
+      <c r="D16" t="n">
+        <v>95</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-01T11:04:48+02:00</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1749</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1654</v>
+      </c>
+      <c r="D17" t="n">
+        <v>95</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>-25</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Price check: EUR 1766 (available) 2026-10-05
Co-authored-by: woutergroeneweg-blip <woutergroeneweg-blip@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/prices.xlsx
+++ b/prices.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price History" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Price History" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -138,14 +138,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -168,26 +167,26 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <cat>
             <numRef>
-              <f>'Price History'!$A$2</f>
+              <f>'Price History'!$A$2:$A$18</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Price History'!$B$2</f>
+              <f>'Price History'!$B$2:$B$18</f>
             </numRef>
           </val>
         </ser>
@@ -203,8 +202,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -230,8 +229,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -257,7 +256,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -272,9 +271,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -572,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -658,6 +657,550 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>Baseline from Roompot confirmation screenshot; replace/extend with live automation runs</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-01T11:09:16+02:00</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1809</v>
+      </c>
+      <c r="D3" t="n">
+        <v>95</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>-17</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-05T11:06:27+02:00</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1797</v>
+      </c>
+      <c r="D4" t="n">
+        <v>95</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>-12</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-09T11:06:32+02:00</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1910</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1815</v>
+      </c>
+      <c r="D5" t="n">
+        <v>95</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>+18</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-13T11:11:58+02:00</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1921</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1826</v>
+      </c>
+      <c r="D6" t="n">
+        <v>95</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>+11</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-21T11:05:50+02:00</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1745</v>
+      </c>
+      <c r="D7" t="n">
+        <v>95</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>-81</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-25T11:07:23+02:00</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1844</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1749</v>
+      </c>
+      <c r="D8" t="n">
+        <v>95</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>+4</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-29T11:15:29+02:00</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1876</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1781</v>
+      </c>
+      <c r="D9" t="n">
+        <v>95</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>+32</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-01T11:07:41+02:00</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1767</v>
+      </c>
+      <c r="D10" t="n">
+        <v>95</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>-14</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-05T11:06:59+02:00</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1682</v>
+      </c>
+      <c r="D11" t="n">
+        <v>95</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>-85</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-09T11:08:10+02:00</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1666</v>
+      </c>
+      <c r="D12" t="n">
+        <v>95</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>-16</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:14:39+02:00</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D13" t="n">
+        <v>95</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>+12</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-21T11:06:05+02:00</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D14" t="n">
+        <v>95</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:09:00+02:00</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1674</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1579</v>
+      </c>
+      <c r="D15" t="n">
+        <v>95</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>-99</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29T11:05:58+02:00</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1774</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1679</v>
+      </c>
+      <c r="D16" t="n">
+        <v>95</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-01T11:04:48+02:00</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1749</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1654</v>
+      </c>
+      <c r="D17" t="n">
+        <v>95</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>-25</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-05T11:05:39+02:00</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1766</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1671</v>
+      </c>
+      <c r="D18" t="n">
+        <v>95</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>+17</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Price check: EUR 1629 (available) 2026-10-09
Co-authored-by: woutergroeneweg-blip <woutergroeneweg-blip@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/prices.xlsx
+++ b/prices.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price History" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Price History" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -138,14 +138,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -168,26 +167,26 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <cat>
             <numRef>
-              <f>'Price History'!$A$2</f>
+              <f>'Price History'!$A$2:$A$19</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Price History'!$B$2</f>
+              <f>'Price History'!$B$2:$B$19</f>
             </numRef>
           </val>
         </ser>
@@ -203,8 +202,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -230,8 +229,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -257,7 +256,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -272,9 +271,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -572,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -658,6 +657,584 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>Baseline from Roompot confirmation screenshot; replace/extend with live automation runs</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-01T11:09:16+02:00</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1809</v>
+      </c>
+      <c r="D3" t="n">
+        <v>95</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>-17</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-05T11:06:27+02:00</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1797</v>
+      </c>
+      <c r="D4" t="n">
+        <v>95</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>-12</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-09T11:06:32+02:00</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1910</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1815</v>
+      </c>
+      <c r="D5" t="n">
+        <v>95</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>+18</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-13T11:11:58+02:00</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1921</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1826</v>
+      </c>
+      <c r="D6" t="n">
+        <v>95</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>+11</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-21T11:05:50+02:00</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1745</v>
+      </c>
+      <c r="D7" t="n">
+        <v>95</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>-81</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-25T11:07:23+02:00</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1844</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1749</v>
+      </c>
+      <c r="D8" t="n">
+        <v>95</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>+4</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-29T11:15:29+02:00</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1876</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1781</v>
+      </c>
+      <c r="D9" t="n">
+        <v>95</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>+32</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-01T11:07:41+02:00</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1767</v>
+      </c>
+      <c r="D10" t="n">
+        <v>95</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>-14</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-05T11:06:59+02:00</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1682</v>
+      </c>
+      <c r="D11" t="n">
+        <v>95</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>-85</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-09T11:08:10+02:00</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1666</v>
+      </c>
+      <c r="D12" t="n">
+        <v>95</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>-16</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:14:39+02:00</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D13" t="n">
+        <v>95</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>+12</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-21T11:06:05+02:00</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D14" t="n">
+        <v>95</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:09:00+02:00</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1674</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1579</v>
+      </c>
+      <c r="D15" t="n">
+        <v>95</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>-99</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29T11:05:58+02:00</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1774</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1679</v>
+      </c>
+      <c r="D16" t="n">
+        <v>95</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-01T11:04:48+02:00</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1749</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1654</v>
+      </c>
+      <c r="D17" t="n">
+        <v>95</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>-25</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-05T11:05:39+02:00</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1766</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1671</v>
+      </c>
+      <c r="D18" t="n">
+        <v>95</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>+17</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-09T11:08:05+02:00</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1629</v>
+      </c>
+      <c r="C19" t="n">
+        <v>1534</v>
+      </c>
+      <c r="D19" t="n">
+        <v>95</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>-137</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>1629</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Price check: EUR 1599 (available) 2026-10-13
Co-authored-by: woutergroeneweg-blip <woutergroeneweg-blip@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/prices.xlsx
+++ b/prices.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price History" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Price History" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -138,14 +138,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -168,26 +167,26 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <cat>
             <numRef>
-              <f>'Price History'!$A$2</f>
+              <f>'Price History'!$A$2:$A$20</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Price History'!$B$2</f>
+              <f>'Price History'!$B$2:$B$20</f>
             </numRef>
           </val>
         </ser>
@@ -203,8 +202,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -230,8 +229,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -257,7 +256,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -272,9 +271,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -572,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -658,6 +657,618 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>Baseline from Roompot confirmation screenshot; replace/extend with live automation runs</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-01T11:09:16+02:00</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1809</v>
+      </c>
+      <c r="D3" t="n">
+        <v>95</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>-17</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-05T11:06:27+02:00</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1797</v>
+      </c>
+      <c r="D4" t="n">
+        <v>95</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>-12</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-09T11:06:32+02:00</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1910</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1815</v>
+      </c>
+      <c r="D5" t="n">
+        <v>95</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>+18</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-13T11:11:58+02:00</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1921</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1826</v>
+      </c>
+      <c r="D6" t="n">
+        <v>95</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>+11</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-21T11:05:50+02:00</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1745</v>
+      </c>
+      <c r="D7" t="n">
+        <v>95</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>-81</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-25T11:07:23+02:00</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1844</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1749</v>
+      </c>
+      <c r="D8" t="n">
+        <v>95</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>+4</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-29T11:15:29+02:00</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1876</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1781</v>
+      </c>
+      <c r="D9" t="n">
+        <v>95</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>+32</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-01T11:07:41+02:00</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1767</v>
+      </c>
+      <c r="D10" t="n">
+        <v>95</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>-14</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-05T11:06:59+02:00</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1682</v>
+      </c>
+      <c r="D11" t="n">
+        <v>95</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>-85</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-09T11:08:10+02:00</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1666</v>
+      </c>
+      <c r="D12" t="n">
+        <v>95</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>-16</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:14:39+02:00</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D13" t="n">
+        <v>95</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>+12</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-21T11:06:05+02:00</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D14" t="n">
+        <v>95</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:09:00+02:00</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1674</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1579</v>
+      </c>
+      <c r="D15" t="n">
+        <v>95</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>-99</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29T11:05:58+02:00</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1774</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1679</v>
+      </c>
+      <c r="D16" t="n">
+        <v>95</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-01T11:04:48+02:00</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1749</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1654</v>
+      </c>
+      <c r="D17" t="n">
+        <v>95</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>-25</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-05T11:05:39+02:00</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1766</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1671</v>
+      </c>
+      <c r="D18" t="n">
+        <v>95</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>+17</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-09T11:08:05+02:00</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1629</v>
+      </c>
+      <c r="C19" t="n">
+        <v>1534</v>
+      </c>
+      <c r="D19" t="n">
+        <v>95</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>-137</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>1629</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-13T11:07:51+02:00</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1599</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1504</v>
+      </c>
+      <c r="D20" t="n">
+        <v>95</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>-30</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>1599</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Price check: EUR 1523 (available) 2026-10-17
Co-authored-by: woutergroeneweg-blip <woutergroeneweg-blip@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/prices.xlsx
+++ b/prices.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price History" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Price History" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -138,14 +138,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -168,26 +167,26 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <cat>
             <numRef>
-              <f>'Price History'!$A$2</f>
+              <f>'Price History'!$A$2:$A$21</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Price History'!$B$2</f>
+              <f>'Price History'!$B$2:$B$21</f>
             </numRef>
           </val>
         </ser>
@@ -203,8 +202,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -230,8 +229,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -257,7 +256,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -272,9 +271,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -572,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -658,6 +657,652 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>Baseline from Roompot confirmation screenshot; replace/extend with live automation runs</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-01T11:09:16+02:00</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1809</v>
+      </c>
+      <c r="D3" t="n">
+        <v>95</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>-17</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-05T11:06:27+02:00</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1797</v>
+      </c>
+      <c r="D4" t="n">
+        <v>95</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>-12</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-09T11:06:32+02:00</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1910</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1815</v>
+      </c>
+      <c r="D5" t="n">
+        <v>95</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>+18</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-13T11:11:58+02:00</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1921</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1826</v>
+      </c>
+      <c r="D6" t="n">
+        <v>95</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>+11</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-21T11:05:50+02:00</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1745</v>
+      </c>
+      <c r="D7" t="n">
+        <v>95</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>-81</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-25T11:07:23+02:00</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1844</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1749</v>
+      </c>
+      <c r="D8" t="n">
+        <v>95</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>+4</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-29T11:15:29+02:00</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1876</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1781</v>
+      </c>
+      <c r="D9" t="n">
+        <v>95</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>+32</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-01T11:07:41+02:00</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1767</v>
+      </c>
+      <c r="D10" t="n">
+        <v>95</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>-14</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-05T11:06:59+02:00</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1682</v>
+      </c>
+      <c r="D11" t="n">
+        <v>95</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>-85</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-09T11:08:10+02:00</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1666</v>
+      </c>
+      <c r="D12" t="n">
+        <v>95</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>-16</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:14:39+02:00</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D13" t="n">
+        <v>95</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>+12</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-21T11:06:05+02:00</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D14" t="n">
+        <v>95</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:09:00+02:00</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1674</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1579</v>
+      </c>
+      <c r="D15" t="n">
+        <v>95</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>-99</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29T11:05:58+02:00</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1774</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1679</v>
+      </c>
+      <c r="D16" t="n">
+        <v>95</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-01T11:04:48+02:00</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1749</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1654</v>
+      </c>
+      <c r="D17" t="n">
+        <v>95</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>-25</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-05T11:05:39+02:00</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1766</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1671</v>
+      </c>
+      <c r="D18" t="n">
+        <v>95</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>+17</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-09T11:08:05+02:00</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1629</v>
+      </c>
+      <c r="C19" t="n">
+        <v>1534</v>
+      </c>
+      <c r="D19" t="n">
+        <v>95</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>-137</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>1629</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-13T11:07:51+02:00</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1599</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1504</v>
+      </c>
+      <c r="D20" t="n">
+        <v>95</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>-30</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>1599</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:09:27+02:00</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1523</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1428</v>
+      </c>
+      <c r="D21" t="n">
+        <v>95</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>-76</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>1523</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Price check: EUR 1498 (available) 2026-10-21
Co-authored-by: woutergroeneweg-blip <woutergroeneweg-blip@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/prices.xlsx
+++ b/prices.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price History" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Price History" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -138,14 +138,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -168,26 +167,26 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <cat>
             <numRef>
-              <f>'Price History'!$A$2</f>
+              <f>'Price History'!$A$2:$A$22</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Price History'!$B$2</f>
+              <f>'Price History'!$B$2:$B$22</f>
             </numRef>
           </val>
         </ser>
@@ -203,8 +202,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -230,8 +229,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -257,7 +256,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -272,9 +271,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -572,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -658,6 +657,686 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>Baseline from Roompot confirmation screenshot; replace/extend with live automation runs</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-01T11:09:16+02:00</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1809</v>
+      </c>
+      <c r="D3" t="n">
+        <v>95</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>-17</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-05T11:06:27+02:00</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1797</v>
+      </c>
+      <c r="D4" t="n">
+        <v>95</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>-12</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-09T11:06:32+02:00</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1910</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1815</v>
+      </c>
+      <c r="D5" t="n">
+        <v>95</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>+18</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-13T11:11:58+02:00</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1921</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1826</v>
+      </c>
+      <c r="D6" t="n">
+        <v>95</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>+11</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-21T11:05:50+02:00</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1745</v>
+      </c>
+      <c r="D7" t="n">
+        <v>95</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>-81</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-25T11:07:23+02:00</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1844</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1749</v>
+      </c>
+      <c r="D8" t="n">
+        <v>95</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>+4</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-29T11:15:29+02:00</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1876</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1781</v>
+      </c>
+      <c r="D9" t="n">
+        <v>95</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>+32</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-01T11:07:41+02:00</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1767</v>
+      </c>
+      <c r="D10" t="n">
+        <v>95</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>-14</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-05T11:06:59+02:00</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1682</v>
+      </c>
+      <c r="D11" t="n">
+        <v>95</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>-85</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-09T11:08:10+02:00</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1666</v>
+      </c>
+      <c r="D12" t="n">
+        <v>95</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>-16</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:14:39+02:00</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D13" t="n">
+        <v>95</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>+12</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-21T11:06:05+02:00</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D14" t="n">
+        <v>95</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:09:00+02:00</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1674</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1579</v>
+      </c>
+      <c r="D15" t="n">
+        <v>95</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>-99</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29T11:05:58+02:00</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1774</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1679</v>
+      </c>
+      <c r="D16" t="n">
+        <v>95</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-01T11:04:48+02:00</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1749</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1654</v>
+      </c>
+      <c r="D17" t="n">
+        <v>95</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>-25</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-05T11:05:39+02:00</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1766</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1671</v>
+      </c>
+      <c r="D18" t="n">
+        <v>95</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>+17</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-09T11:08:05+02:00</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1629</v>
+      </c>
+      <c r="C19" t="n">
+        <v>1534</v>
+      </c>
+      <c r="D19" t="n">
+        <v>95</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>-137</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>1629</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-13T11:07:51+02:00</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1599</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1504</v>
+      </c>
+      <c r="D20" t="n">
+        <v>95</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>-30</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>1599</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:09:27+02:00</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1523</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1428</v>
+      </c>
+      <c r="D21" t="n">
+        <v>95</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>-76</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>1523</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10-21T11:04:44+02:00</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1498</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1403</v>
+      </c>
+      <c r="D22" t="n">
+        <v>95</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>-25</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>1498</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Price check: EUR 1596 (available) 2026-10-25
Co-authored-by: woutergroeneweg-blip <woutergroeneweg-blip@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/prices.xlsx
+++ b/prices.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price History" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Price History" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -138,14 +138,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -168,26 +167,26 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <cat>
             <numRef>
-              <f>'Price History'!$A$2</f>
+              <f>'Price History'!$A$2:$A$23</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Price History'!$B$2</f>
+              <f>'Price History'!$B$2:$B$23</f>
             </numRef>
           </val>
         </ser>
@@ -203,8 +202,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -230,8 +229,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -257,7 +256,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -272,9 +271,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -572,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -658,6 +657,720 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>Baseline from Roompot confirmation screenshot; replace/extend with live automation runs</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-01T11:09:16+02:00</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1809</v>
+      </c>
+      <c r="D3" t="n">
+        <v>95</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>-17</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-05T11:06:27+02:00</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1797</v>
+      </c>
+      <c r="D4" t="n">
+        <v>95</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>-12</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-09T11:06:32+02:00</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1910</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1815</v>
+      </c>
+      <c r="D5" t="n">
+        <v>95</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>+18</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-13T11:11:58+02:00</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1921</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1826</v>
+      </c>
+      <c r="D6" t="n">
+        <v>95</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>+11</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-21T11:05:50+02:00</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1745</v>
+      </c>
+      <c r="D7" t="n">
+        <v>95</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>-81</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-25T11:07:23+02:00</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1844</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1749</v>
+      </c>
+      <c r="D8" t="n">
+        <v>95</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>+4</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-29T11:15:29+02:00</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1876</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1781</v>
+      </c>
+      <c r="D9" t="n">
+        <v>95</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>+32</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-01T11:07:41+02:00</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1767</v>
+      </c>
+      <c r="D10" t="n">
+        <v>95</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>-14</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-05T11:06:59+02:00</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1682</v>
+      </c>
+      <c r="D11" t="n">
+        <v>95</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>-85</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-09T11:08:10+02:00</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1666</v>
+      </c>
+      <c r="D12" t="n">
+        <v>95</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>-16</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:14:39+02:00</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D13" t="n">
+        <v>95</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>+12</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-21T11:06:05+02:00</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D14" t="n">
+        <v>95</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:09:00+02:00</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1674</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1579</v>
+      </c>
+      <c r="D15" t="n">
+        <v>95</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>-99</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29T11:05:58+02:00</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1774</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1679</v>
+      </c>
+      <c r="D16" t="n">
+        <v>95</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-01T11:04:48+02:00</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1749</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1654</v>
+      </c>
+      <c r="D17" t="n">
+        <v>95</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>-25</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-05T11:05:39+02:00</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1766</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1671</v>
+      </c>
+      <c r="D18" t="n">
+        <v>95</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>+17</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-09T11:08:05+02:00</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1629</v>
+      </c>
+      <c r="C19" t="n">
+        <v>1534</v>
+      </c>
+      <c r="D19" t="n">
+        <v>95</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>-137</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>1629</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-13T11:07:51+02:00</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1599</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1504</v>
+      </c>
+      <c r="D20" t="n">
+        <v>95</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>-30</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>1599</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:09:27+02:00</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1523</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1428</v>
+      </c>
+      <c r="D21" t="n">
+        <v>95</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>-76</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>1523</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10-21T11:04:44+02:00</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1498</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1403</v>
+      </c>
+      <c r="D22" t="n">
+        <v>95</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>-25</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>1498</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-25T10:03:09+01:00</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1596</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1501</v>
+      </c>
+      <c r="D23" t="n">
+        <v>95</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>+98</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>1498</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Price check: EUR 1666 (available) 2026-10-29
Co-authored-by: woutergroeneweg-blip <woutergroeneweg-blip@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/prices.xlsx
+++ b/prices.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price History" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Price History" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -138,14 +138,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -168,26 +167,26 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <cat>
             <numRef>
-              <f>'Price History'!$A$2</f>
+              <f>'Price History'!$A$2:$A$24</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Price History'!$B$2</f>
+              <f>'Price History'!$B$2:$B$24</f>
             </numRef>
           </val>
         </ser>
@@ -203,8 +202,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -230,8 +229,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -257,7 +256,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -272,9 +271,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -572,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -658,6 +657,754 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>Baseline from Roompot confirmation screenshot; replace/extend with live automation runs</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-01T11:09:16+02:00</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1809</v>
+      </c>
+      <c r="D3" t="n">
+        <v>95</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>-17</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-05T11:06:27+02:00</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1797</v>
+      </c>
+      <c r="D4" t="n">
+        <v>95</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>-12</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-09T11:06:32+02:00</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1910</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1815</v>
+      </c>
+      <c r="D5" t="n">
+        <v>95</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>+18</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-13T11:11:58+02:00</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1921</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1826</v>
+      </c>
+      <c r="D6" t="n">
+        <v>95</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>+11</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-21T11:05:50+02:00</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1745</v>
+      </c>
+      <c r="D7" t="n">
+        <v>95</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>-81</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-25T11:07:23+02:00</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1844</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1749</v>
+      </c>
+      <c r="D8" t="n">
+        <v>95</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>+4</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-29T11:15:29+02:00</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1876</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1781</v>
+      </c>
+      <c r="D9" t="n">
+        <v>95</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>+32</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-01T11:07:41+02:00</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1767</v>
+      </c>
+      <c r="D10" t="n">
+        <v>95</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>-14</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-05T11:06:59+02:00</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1682</v>
+      </c>
+      <c r="D11" t="n">
+        <v>95</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>-85</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-09T11:08:10+02:00</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1666</v>
+      </c>
+      <c r="D12" t="n">
+        <v>95</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>-16</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:14:39+02:00</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D13" t="n">
+        <v>95</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>+12</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-21T11:06:05+02:00</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D14" t="n">
+        <v>95</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:09:00+02:00</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1674</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1579</v>
+      </c>
+      <c r="D15" t="n">
+        <v>95</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>-99</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29T11:05:58+02:00</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1774</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1679</v>
+      </c>
+      <c r="D16" t="n">
+        <v>95</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-01T11:04:48+02:00</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1749</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1654</v>
+      </c>
+      <c r="D17" t="n">
+        <v>95</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>-25</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-05T11:05:39+02:00</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1766</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1671</v>
+      </c>
+      <c r="D18" t="n">
+        <v>95</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>+17</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-09T11:08:05+02:00</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1629</v>
+      </c>
+      <c r="C19" t="n">
+        <v>1534</v>
+      </c>
+      <c r="D19" t="n">
+        <v>95</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>-137</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>1629</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-13T11:07:51+02:00</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1599</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1504</v>
+      </c>
+      <c r="D20" t="n">
+        <v>95</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>-30</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>1599</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:09:27+02:00</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1523</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1428</v>
+      </c>
+      <c r="D21" t="n">
+        <v>95</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>-76</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>1523</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10-21T11:04:44+02:00</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1498</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1403</v>
+      </c>
+      <c r="D22" t="n">
+        <v>95</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>-25</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>1498</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-25T10:03:09+01:00</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1596</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1501</v>
+      </c>
+      <c r="D23" t="n">
+        <v>95</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>+98</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>1498</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-10-29T10:13:05+01:00</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1666</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1571</v>
+      </c>
+      <c r="D24" t="n">
+        <v>95</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>+70</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>1498</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Price check: EUR 1661 (available) 2026-11-01
Co-authored-by: woutergroeneweg-blip <woutergroeneweg-blip@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/prices.xlsx
+++ b/prices.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Price History" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Price History" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -138,14 +138,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -168,26 +167,26 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <cat>
             <numRef>
-              <f>'Price History'!$A$2</f>
+              <f>'Price History'!$A$2:$A$25</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Price History'!$B$2</f>
+              <f>'Price History'!$B$2:$B$25</f>
             </numRef>
           </val>
         </ser>
@@ -203,8 +202,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -230,8 +229,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -257,7 +256,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>9</col>
@@ -272,9 +271,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -572,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -658,6 +657,788 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>Baseline from Roompot confirmation screenshot; replace/extend with live automation runs</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-01T11:09:16+02:00</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1809</v>
+      </c>
+      <c r="D3" t="n">
+        <v>95</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>-17</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-05T11:06:27+02:00</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1797</v>
+      </c>
+      <c r="D4" t="n">
+        <v>95</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>-12</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-09T11:06:32+02:00</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1910</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1815</v>
+      </c>
+      <c r="D5" t="n">
+        <v>95</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>+18</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-13T11:11:58+02:00</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1921</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1826</v>
+      </c>
+      <c r="D6" t="n">
+        <v>95</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>+11</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1892</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-21T11:05:50+02:00</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1745</v>
+      </c>
+      <c r="D7" t="n">
+        <v>95</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>-81</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-25T11:07:23+02:00</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1844</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1749</v>
+      </c>
+      <c r="D8" t="n">
+        <v>95</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>+4</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-29T11:15:29+02:00</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1876</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1781</v>
+      </c>
+      <c r="D9" t="n">
+        <v>95</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>+32</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-01T11:07:41+02:00</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1862</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1767</v>
+      </c>
+      <c r="D10" t="n">
+        <v>95</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>-14</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>1840</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-05T11:06:59+02:00</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1682</v>
+      </c>
+      <c r="D11" t="n">
+        <v>95</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>-85</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1777</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-09T11:08:10+02:00</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1666</v>
+      </c>
+      <c r="D12" t="n">
+        <v>95</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>-16</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-17T11:14:39+02:00</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D13" t="n">
+        <v>95</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>+12</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-21T11:06:05+02:00</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1773</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D14" t="n">
+        <v>95</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1761</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:09:00+02:00</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1674</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1579</v>
+      </c>
+      <c r="D15" t="n">
+        <v>95</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>-99</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29T11:05:58+02:00</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1774</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1679</v>
+      </c>
+      <c r="D16" t="n">
+        <v>95</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>+100</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-01T11:04:48+02:00</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1749</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1654</v>
+      </c>
+      <c r="D17" t="n">
+        <v>95</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>-25</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-05T11:05:39+02:00</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1766</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1671</v>
+      </c>
+      <c r="D18" t="n">
+        <v>95</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>+17</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>1674</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-09T11:08:05+02:00</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1629</v>
+      </c>
+      <c r="C19" t="n">
+        <v>1534</v>
+      </c>
+      <c r="D19" t="n">
+        <v>95</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>-137</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>1629</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-13T11:07:51+02:00</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1599</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1504</v>
+      </c>
+      <c r="D20" t="n">
+        <v>95</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>-30</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>1599</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-10-17T11:09:27+02:00</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1523</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1428</v>
+      </c>
+      <c r="D21" t="n">
+        <v>95</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>-76</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>1523</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10-21T11:04:44+02:00</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1498</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1403</v>
+      </c>
+      <c r="D22" t="n">
+        <v>95</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>-25</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>1498</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-25T10:03:09+01:00</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1596</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1501</v>
+      </c>
+      <c r="D23" t="n">
+        <v>95</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>+98</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>1498</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-10-29T10:13:05+01:00</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1666</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1571</v>
+      </c>
+      <c r="D24" t="n">
+        <v>95</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>+70</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>1498</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-11-01T10:09:31+01:00</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1661</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1566</v>
+      </c>
+      <c r="D25" t="n">
+        <v>95</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>available</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>-5</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>1498</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>scheduled automation run</t>
         </is>
       </c>
     </row>

</xml_diff>